<commit_message>
chore: mise à jour automatique des données (2026-10-14)
</commit_message>
<xml_diff>
--- a/tests/fixtures/finances_sociales/classeur_2024.xlsx
+++ b/tests/fixtures/finances_sociales/classeur_2024.xlsx
@@ -1140,6 +1140,151 @@
 </sst>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="10" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="36.6328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6328125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.90625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="30" customFormat="1" ht="10.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="28"/>
+      <c r="B1" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="10.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="9">
+        <v>27097.8</v>
+      </c>
+      <c r="C2" s="9">
+        <v>27918.1</v>
+      </c>
+      <c r="D2" s="9">
+        <v>29946</v>
+      </c>
+      <c r="E2" s="9">
+        <v>31991.8</v>
+      </c>
+      <c r="F2" s="9">
+        <v>33137.4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="2">
+        <v>401</v>
+      </c>
+      <c r="C3" s="2">
+        <v>432</v>
+      </c>
+      <c r="D3" s="2">
+        <v>546.20000000000005</v>
+      </c>
+      <c r="E3" s="2">
+        <v>587.20000000000005</v>
+      </c>
+      <c r="F3" s="54">
+        <v>33137.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="2">
+        <v>26696.799999999999</v>
+      </c>
+      <c r="C4" s="2">
+        <v>27486.1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>29399.8</v>
+      </c>
+      <c r="E4" s="2">
+        <v>31404.6</v>
+      </c>
+      <c r="F4" s="54"/>
+    </row>
+    <row r="5" spans="1:6" ht="10.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="9">
+        <v>759</v>
+      </c>
+      <c r="C5" s="9">
+        <v>816</v>
+      </c>
+      <c r="D5" s="9">
+        <v>883</v>
+      </c>
+      <c r="E5" s="9">
+        <v>940</v>
+      </c>
+      <c r="F5" s="9">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="32">
+        <v>759</v>
+      </c>
+      <c r="C6" s="32">
+        <v>816</v>
+      </c>
+      <c r="D6" s="32">
+        <v>883</v>
+      </c>
+      <c r="E6" s="32">
+        <v>940</v>
+      </c>
+      <c r="F6" s="32">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="A8" s="51" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="36" t="s">
+        <v>350</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F3:F4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:F22"/>
@@ -1533,6 +1678,285 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="F11:F13"/>
+    <mergeCell ref="F3:F4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="10" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="36.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="6" width="10.6328125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="10.90625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="30" customFormat="1" ht="10.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="28"/>
+      <c r="B1" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="10.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="9">
+        <v>168140.19</v>
+      </c>
+      <c r="C2" s="9">
+        <v>160415.21</v>
+      </c>
+      <c r="D2" s="9">
+        <v>155012.51</v>
+      </c>
+      <c r="E2" s="9">
+        <v>156826.63</v>
+      </c>
+      <c r="F2" s="9">
+        <v>161903.31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="2">
+        <v>123855.03</v>
+      </c>
+      <c r="C3" s="2">
+        <v>116623.87</v>
+      </c>
+      <c r="D3" s="2">
+        <v>110735.09</v>
+      </c>
+      <c r="E3" s="2">
+        <v>112840.7</v>
+      </c>
+      <c r="F3" s="53">
+        <v>161856.31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="2">
+        <v>42287.66</v>
+      </c>
+      <c r="C4" s="2">
+        <v>42904.94</v>
+      </c>
+      <c r="D4" s="2">
+        <v>41905.42</v>
+      </c>
+      <c r="E4" s="2">
+        <v>44079.93</v>
+      </c>
+      <c r="F4" s="53"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2">
+        <v>367</v>
+      </c>
+      <c r="D5" s="2">
+        <v>464</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1997.5</v>
+      </c>
+      <c r="C6" s="2">
+        <v>519.4</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1908</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-94</v>
+      </c>
+      <c r="F6" s="2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="10.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="9">
+        <v>176412.64</v>
+      </c>
+      <c r="C7" s="9">
+        <v>167274.81</v>
+      </c>
+      <c r="D7" s="9">
+        <v>160943.39000000001</v>
+      </c>
+      <c r="E7" s="9">
+        <v>167169.47</v>
+      </c>
+      <c r="F7" s="9">
+        <v>172927</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1060</v>
+      </c>
+      <c r="C8" s="2">
+        <v>849</v>
+      </c>
+      <c r="D8" s="2">
+        <v>618</v>
+      </c>
+      <c r="E8" s="2">
+        <v>566</v>
+      </c>
+      <c r="F8" s="2">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="2">
+        <v>7132</v>
+      </c>
+      <c r="C9" s="2">
+        <v>7148</v>
+      </c>
+      <c r="D9" s="2">
+        <v>7237</v>
+      </c>
+      <c r="E9" s="2">
+        <v>7391</v>
+      </c>
+      <c r="F9" s="2">
+        <v>7537</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="2">
+        <v>43483</v>
+      </c>
+      <c r="C10" s="2">
+        <v>43660</v>
+      </c>
+      <c r="D10" s="2">
+        <v>45224</v>
+      </c>
+      <c r="E10" s="2">
+        <v>46847</v>
+      </c>
+      <c r="F10" s="2">
+        <v>49837</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="2">
+        <v>11027.19</v>
+      </c>
+      <c r="C11" s="2">
+        <v>8399.42</v>
+      </c>
+      <c r="D11" s="2">
+        <v>7193.74</v>
+      </c>
+      <c r="E11" s="2">
+        <v>5534.15</v>
+      </c>
+      <c r="F11" s="2">
+        <v>5878.71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="2">
+        <v>112896.26</v>
+      </c>
+      <c r="C12" s="2">
+        <v>106383.57</v>
+      </c>
+      <c r="D12" s="2">
+        <v>99866.89</v>
+      </c>
+      <c r="E12" s="2">
+        <v>105977.27</v>
+      </c>
+      <c r="F12" s="2">
+        <v>108309.43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="32">
+        <v>814.19</v>
+      </c>
+      <c r="C13" s="32">
+        <v>834.82</v>
+      </c>
+      <c r="D13" s="32">
+        <v>803.76</v>
+      </c>
+      <c r="E13" s="32">
+        <v>854.05</v>
+      </c>
+      <c r="F13" s="32">
+        <v>904.86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="A15" s="51" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="36" t="s">
+        <v>350</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
     <mergeCell ref="F3:F4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5158,4 +5582,247 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="10" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="36.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.90625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="30" customFormat="1" ht="10.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="28"/>
+      <c r="B1" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="10.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="9">
+        <v>49714.22</v>
+      </c>
+      <c r="C2" s="9">
+        <v>53080.38</v>
+      </c>
+      <c r="D2" s="9">
+        <v>55400</v>
+      </c>
+      <c r="E2" s="9">
+        <v>57438.98</v>
+      </c>
+      <c r="F2" s="9">
+        <v>60162.82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="2">
+        <v>32758.22</v>
+      </c>
+      <c r="C3" s="2">
+        <v>33687.94</v>
+      </c>
+      <c r="D3" s="2">
+        <v>34849</v>
+      </c>
+      <c r="E3" s="2">
+        <v>35887.120000000003</v>
+      </c>
+      <c r="F3" s="53">
+        <v>60130.46</v>
+      </c>
+      <c r="G3" s="31"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="2">
+        <v>16922.099999999999</v>
+      </c>
+      <c r="C4" s="2">
+        <v>19336.12</v>
+      </c>
+      <c r="D4" s="2">
+        <v>20518.080000000002</v>
+      </c>
+      <c r="E4" s="2">
+        <v>21519.42</v>
+      </c>
+      <c r="F4" s="53"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="2">
+        <v>33.9</v>
+      </c>
+      <c r="C5" s="2">
+        <v>56.32</v>
+      </c>
+      <c r="D5" s="2">
+        <v>32.92</v>
+      </c>
+      <c r="E5" s="2">
+        <v>32.44</v>
+      </c>
+      <c r="F5" s="2">
+        <v>32.36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="10.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="9">
+        <v>58518.59</v>
+      </c>
+      <c r="C6" s="9">
+        <v>63008.76</v>
+      </c>
+      <c r="D6" s="9">
+        <v>64680.14</v>
+      </c>
+      <c r="E6" s="9">
+        <v>69285.09</v>
+      </c>
+      <c r="F6" s="9">
+        <v>73236.53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="2">
+        <v>962.61</v>
+      </c>
+      <c r="C7" s="2">
+        <v>983.03</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1031.0999999999999</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1072.69</v>
+      </c>
+      <c r="F7" s="53">
+        <v>51174.04</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="2">
+        <v>962.61</v>
+      </c>
+      <c r="C8" s="2">
+        <v>983.03</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1031.0999999999999</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1072.69</v>
+      </c>
+      <c r="F8" s="53"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="2">
+        <v>38577.120000000003</v>
+      </c>
+      <c r="C9" s="2">
+        <v>41926.9</v>
+      </c>
+      <c r="D9" s="2">
+        <v>42126.46</v>
+      </c>
+      <c r="E9" s="2">
+        <v>45696.63</v>
+      </c>
+      <c r="F9" s="53"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="2">
+        <v>17220.45</v>
+      </c>
+      <c r="C10" s="2">
+        <v>18345.189999999999</v>
+      </c>
+      <c r="D10" s="2">
+        <v>19534.62</v>
+      </c>
+      <c r="E10" s="2">
+        <v>20457.59</v>
+      </c>
+      <c r="F10" s="2">
+        <v>20958.330000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="5">
+        <v>795.8</v>
+      </c>
+      <c r="C11" s="5">
+        <v>770.61</v>
+      </c>
+      <c r="D11" s="5">
+        <v>956.86</v>
+      </c>
+      <c r="E11" s="5">
+        <v>985.49</v>
+      </c>
+      <c r="F11" s="5">
+        <v>1104.1600000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A13" s="51" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="36" t="s">
+        <v>350</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="F7:F9"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>